<commit_message>
Everything is so convoluted...but somehow better.
</commit_message>
<xml_diff>
--- a/WorkBot/refactor/data/orders/Coca-Cola/Coca-Cola_Collegetown_2025-10-17.xlsx
+++ b/WorkBot/refactor/data/orders/Coca-Cola/Coca-Cola_Collegetown_2025-10-17.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>77.12</t>
+          <t>154.24</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>26.46</t>
+          <t>52.92</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>65.80</t>
+          <t>98.70</t>
         </is>
       </c>
     </row>

</xml_diff>